<commit_message>
Fix scene data quality anomalies
</commit_message>
<xml_diff>
--- a/ball_at_opponent_normalized_prototype_v2_executable.xlsx
+++ b/ball_at_opponent_normalized_prototype_v2_executable.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="normalized_opponent_scenes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="verification" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="semantic_rules" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="normalized_opponent_scenes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="verification" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="semantic_rules" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3340,7 +3340,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>держит мяч...</t>
+          <t>Держит мяч под давлением</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Соперник находится в нашей штрафной . Соперник: держит мяч.... Персонаж находится перед своей штрафной лицом к чужим воротам.</t>
+          <t>Соперник находится в нашей штрафной. Соперник: держит мяч под давлением. Персонаж находится перед своей штрафной лицом к чужим воротам.</t>
         </is>
       </c>
     </row>
@@ -3434,7 +3434,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>держит мяч...</t>
+          <t>Держит мяч под давлением</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Соперник находится в нашей штрафной . Соперник: держит мяч.... Персонаж находится в центре поля лицом к чужим воротам.</t>
+          <t>Соперник находится в нашей штрафной. Соперник: держит мяч под давлением. Персонаж находится в центре поля лицом к чужим воротам.</t>
         </is>
       </c>
     </row>

</xml_diff>